<commit_message>
Modules 00 and 02 gain four new ideas: unlearn the startup advice you got (patents, grants and vanity metrics are not progress), accountability groups of 3 to 7 teams every two weeks with the new Accountability Group Tracker, and skate to where the puck is going (build for the world in five years). Module 06 rebuilt with the Langfuse case, the Show and Build workshop and homework. Updated glossary, rubric, toolkit, legal basics, team stack, tools, archetype guides and frameworks 02 and 06.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PmvC11dUN5PhFNpMi5Rj25
</commit_message>
<xml_diff>
--- a/resources/Student_Toolkit.xlsx
+++ b/resources/Student_Toolkit.xlsx
@@ -14,12 +14,17 @@
     <sheet name="Pain Map" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Experiment Tracker" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Traffic Sources" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="KPI Tracker" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Weekly Reflection" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Self-Assessment" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Evidence Pack" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Revenue Ladder" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Kill Criteria Log" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Use Log" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Pipeline" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Assumptions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bets" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="KPI Tracker" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Weekly Reflection" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Self-Assessment" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Evidence Pack" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Revenue Ladder" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Kill Criteria Log" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Verdict" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -834,7 +839,7 @@
         </is>
       </c>
       <c r="B10" s="19">
-        <f>'KPI Tracker'!C18</f>
+        <f>'KPI Tracker'!C25</f>
         <v/>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -854,7 +859,7 @@
         </is>
       </c>
       <c r="B11" s="19">
-        <f>'KPI Tracker'!C19</f>
+        <f>'KPI Tracker'!C26</f>
         <v/>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1013,6 +1018,1122 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="20" min="1" max="1"/>
+    <col width="40" customWidth="1" style="20" min="2" max="2"/>
+    <col width="20" customWidth="1" style="20" min="3" max="3"/>
+    <col width="12" customWidth="1" style="20" min="4" max="4"/>
+    <col width="30" customWidth="1" style="20" min="5" max="5"/>
+    <col width="12" customWidth="1" style="20" min="6" max="6"/>
+    <col width="30" customWidth="1" style="20" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Module 07. One row per assumption your venture still rests on. Mark it critical or not, known (name the artifact) or assumed. The monkey is critical and unknown, and you test it first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1" s="20">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Area (customer, solution, business)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Critical? (yes, no)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Known (artifact) or assumed</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Monkey? (yes, no)</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Test and line (Kill Criteria Log row)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="20" min="1" max="1"/>
+    <col width="28" customWidth="1" style="20" min="2" max="2"/>
+    <col width="16" customWidth="1" style="20" min="3" max="3"/>
+    <col width="16" customWidth="1" style="20" min="4" max="4"/>
+    <col width="16" customWidth="1" style="20" min="5" max="5"/>
+    <col width="28" customWidth="1" style="20" min="6" max="6"/>
+    <col width="16" customWidth="1" style="20" min="7" max="7"/>
+    <col width="16" customWidth="1" style="20" min="8" max="8"/>
+    <col width="16" customWidth="1" style="20" min="9" max="9"/>
+    <col width="16" customWidth="1" style="20" min="10" max="10"/>
+    <col width="16" customWidth="1" style="20" min="11" max="11"/>
+    <col width="28" customWidth="1" style="20" min="12" max="12"/>
+    <col width="28" customWidth="1" style="20" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>BETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Module 10. One row per request, idea or fix. Write who asked, the driver it should move and the expected effect before you build. Keep only what a paying customer asked for and what deepens the core outcome. Tell the others no, and note the date.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1" s="20">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Date written</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Bet (request, idea or fix)</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Who asked</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Pays? (yes, no)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Driver it should move</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Expected effect, by when (written before building)</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Kept or buried</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Why not now (if buried)</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Now, Next or Later</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="K4" s="28" t="inlineStr">
+        <is>
+          <t>Shipped on</t>
+        </is>
+      </c>
+      <c r="L4" s="28" t="inlineStr">
+        <is>
+          <t>Result against the expected effect</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="inlineStr">
+        <is>
+          <t>Told no on (date, if buried)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:N34"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="25" customWidth="1" style="19" min="1" max="1"/>
+    <col width="8" customWidth="1" style="19" min="2" max="13"/>
+    <col width="13" customWidth="1" style="20" min="13" max="13"/>
+    <col width="13" customWidth="1" style="20" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>KPI TRACKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="20">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>WEEKLY METRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="20">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>M00</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>M02</t>
+        </is>
+      </c>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>M03</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>M04</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="inlineStr">
+        <is>
+          <t>M05</t>
+        </is>
+      </c>
+      <c r="H4" s="32" t="inlineStr">
+        <is>
+          <t>M06</t>
+        </is>
+      </c>
+      <c r="I4" s="32" t="inlineStr">
+        <is>
+          <t>M07</t>
+        </is>
+      </c>
+      <c r="J4" s="32" t="inlineStr">
+        <is>
+          <t>M08</t>
+        </is>
+      </c>
+      <c r="K4" s="32" t="inlineStr">
+        <is>
+          <t>M09</t>
+        </is>
+      </c>
+      <c r="L4" s="32" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="M4" s="32" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="N4" s="32" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="20">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>North Star (your weekly count)</t>
+        </is>
+      </c>
+      <c r="B5" s="34" t="n"/>
+      <c r="C5" s="34" t="n"/>
+      <c r="D5" s="34" t="n"/>
+      <c r="E5" s="34" t="n"/>
+      <c r="F5" s="34" t="n"/>
+      <c r="G5" s="34" t="n"/>
+      <c r="H5" s="34" t="n"/>
+      <c r="I5" s="34" t="n"/>
+      <c r="J5" s="34" t="n"/>
+      <c r="K5" s="34" t="n"/>
+      <c r="L5" s="34" t="n"/>
+      <c r="M5" s="34" t="n"/>
+      <c r="N5" s="34" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="20">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Interviews Conducted</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="n"/>
+      <c r="C6" s="34" t="n"/>
+      <c r="D6" s="34" t="n"/>
+      <c r="E6" s="34" t="n"/>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="34" t="n"/>
+      <c r="H6" s="34" t="n"/>
+      <c r="I6" s="34" t="n"/>
+      <c r="J6" s="34" t="n"/>
+      <c r="K6" s="34" t="n"/>
+      <c r="L6" s="34" t="n"/>
+      <c r="M6" s="34" t="n"/>
+      <c r="N6" s="34" t="n"/>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="20">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Experiments Run</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="n"/>
+      <c r="C7" s="34" t="n"/>
+      <c r="D7" s="34" t="n"/>
+      <c r="E7" s="34" t="n"/>
+      <c r="F7" s="34" t="n"/>
+      <c r="G7" s="34" t="n"/>
+      <c r="H7" s="34" t="n"/>
+      <c r="I7" s="34" t="n"/>
+      <c r="J7" s="34" t="n"/>
+      <c r="K7" s="34" t="n"/>
+      <c r="L7" s="34" t="n"/>
+      <c r="M7" s="34" t="n"/>
+      <c r="N7" s="34" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="20">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>Landing Page Visitors</t>
+        </is>
+      </c>
+      <c r="B8" s="34" t="n"/>
+      <c r="C8" s="34" t="n"/>
+      <c r="D8" s="34" t="n"/>
+      <c r="E8" s="34" t="n"/>
+      <c r="F8" s="34" t="n"/>
+      <c r="G8" s="34" t="n"/>
+      <c r="H8" s="34" t="n"/>
+      <c r="I8" s="34" t="n"/>
+      <c r="J8" s="34" t="n"/>
+      <c r="K8" s="34" t="n"/>
+      <c r="L8" s="34" t="n"/>
+      <c r="M8" s="34" t="n"/>
+      <c r="N8" s="34" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="20">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Sign-ups / Leads</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="n"/>
+      <c r="C9" s="34" t="n"/>
+      <c r="D9" s="34" t="n"/>
+      <c r="E9" s="34" t="n"/>
+      <c r="F9" s="34" t="n"/>
+      <c r="G9" s="34" t="n"/>
+      <c r="H9" s="34" t="n"/>
+      <c r="I9" s="34" t="n"/>
+      <c r="J9" s="34" t="n"/>
+      <c r="K9" s="34" t="n"/>
+      <c r="L9" s="34" t="n"/>
+      <c r="M9" s="34" t="n"/>
+      <c r="N9" s="34" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="20">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Prototype Users</t>
+        </is>
+      </c>
+      <c r="B10" s="34" t="n"/>
+      <c r="C10" s="34" t="n"/>
+      <c r="D10" s="34" t="n"/>
+      <c r="E10" s="34" t="n"/>
+      <c r="F10" s="34" t="n"/>
+      <c r="G10" s="34" t="n"/>
+      <c r="H10" s="34" t="n"/>
+      <c r="I10" s="34" t="n"/>
+      <c r="J10" s="34" t="n"/>
+      <c r="K10" s="34" t="n"/>
+      <c r="L10" s="34" t="n"/>
+      <c r="M10" s="34" t="n"/>
+      <c r="N10" s="34" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="20">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Active Users (weekly)</t>
+        </is>
+      </c>
+      <c r="B11" s="34" t="n"/>
+      <c r="C11" s="34" t="n"/>
+      <c r="D11" s="34" t="n"/>
+      <c r="E11" s="34" t="n"/>
+      <c r="F11" s="34" t="n"/>
+      <c r="G11" s="34" t="n"/>
+      <c r="H11" s="34" t="n"/>
+      <c r="I11" s="34" t="n"/>
+      <c r="J11" s="34" t="n"/>
+      <c r="K11" s="34" t="n"/>
+      <c r="L11" s="34" t="n"/>
+      <c r="M11" s="34" t="n"/>
+      <c r="N11" s="34" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="20">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Activated users (reached the outcome)</t>
+        </is>
+      </c>
+      <c r="B12" s="34" t="n"/>
+      <c r="C12" s="34" t="n"/>
+      <c r="D12" s="34" t="n"/>
+      <c r="E12" s="34" t="n"/>
+      <c r="F12" s="34" t="n"/>
+      <c r="G12" s="34" t="n"/>
+      <c r="H12" s="34" t="n"/>
+      <c r="I12" s="34" t="n"/>
+      <c r="J12" s="34" t="n"/>
+      <c r="K12" s="34" t="n"/>
+      <c r="L12" s="34" t="n"/>
+      <c r="M12" s="34" t="n"/>
+      <c r="N12" s="34" t="n"/>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="20">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Users who came back unprompted</t>
+        </is>
+      </c>
+      <c r="B13" s="34" t="n"/>
+      <c r="C13" s="34" t="n"/>
+      <c r="D13" s="34" t="n"/>
+      <c r="E13" s="34" t="n"/>
+      <c r="F13" s="34" t="n"/>
+      <c r="G13" s="34" t="n"/>
+      <c r="H13" s="34" t="n"/>
+      <c r="I13" s="34" t="n"/>
+      <c r="J13" s="34" t="n"/>
+      <c r="K13" s="34" t="n"/>
+      <c r="L13" s="34" t="n"/>
+      <c r="M13" s="34" t="n"/>
+      <c r="N13" s="34" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Asks made</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="n"/>
+      <c r="C14" s="34" t="n"/>
+      <c r="D14" s="34" t="n"/>
+      <c r="E14" s="34" t="n"/>
+      <c r="F14" s="34" t="n"/>
+      <c r="G14" s="34" t="n"/>
+      <c r="H14" s="34" t="n"/>
+      <c r="I14" s="34" t="n"/>
+      <c r="J14" s="34" t="n"/>
+      <c r="K14" s="34" t="n"/>
+      <c r="L14" s="34" t="n"/>
+      <c r="M14" s="34" t="n"/>
+      <c r="N14" s="34" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="20">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Paying Customers</t>
+        </is>
+      </c>
+      <c r="B15" s="34" t="n"/>
+      <c r="C15" s="34" t="n"/>
+      <c r="D15" s="34" t="n"/>
+      <c r="E15" s="34" t="n"/>
+      <c r="F15" s="34" t="n"/>
+      <c r="G15" s="34" t="n"/>
+      <c r="H15" s="34" t="n"/>
+      <c r="I15" s="34" t="n"/>
+      <c r="J15" s="34" t="n"/>
+      <c r="K15" s="34" t="n"/>
+      <c r="L15" s="34" t="n"/>
+      <c r="M15" s="34" t="n"/>
+      <c r="N15" s="34" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="20">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Payments inside the product</t>
+        </is>
+      </c>
+      <c r="B16" s="34" t="n"/>
+      <c r="C16" s="34" t="n"/>
+      <c r="D16" s="34" t="n"/>
+      <c r="E16" s="34" t="n"/>
+      <c r="F16" s="34" t="n"/>
+      <c r="G16" s="34" t="n"/>
+      <c r="H16" s="34" t="n"/>
+      <c r="I16" s="34" t="n"/>
+      <c r="J16" s="34" t="n"/>
+      <c r="K16" s="34" t="n"/>
+      <c r="L16" s="34" t="n"/>
+      <c r="M16" s="34" t="n"/>
+      <c r="N16" s="34" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="20">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Repeat customers</t>
+        </is>
+      </c>
+      <c r="B17" s="34" t="n"/>
+      <c r="C17" s="34" t="n"/>
+      <c r="D17" s="34" t="n"/>
+      <c r="E17" s="34" t="n"/>
+      <c r="F17" s="34" t="n"/>
+      <c r="G17" s="34" t="n"/>
+      <c r="H17" s="34" t="n"/>
+      <c r="I17" s="34" t="n"/>
+      <c r="J17" s="34" t="n"/>
+      <c r="K17" s="34" t="n"/>
+      <c r="L17" s="34" t="n"/>
+      <c r="M17" s="34" t="n"/>
+      <c r="N17" s="34" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="20">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>Very disappointed, of n asked</t>
+        </is>
+      </c>
+      <c r="B18" s="34" t="n"/>
+      <c r="C18" s="34" t="n"/>
+      <c r="D18" s="34" t="n"/>
+      <c r="E18" s="34" t="n"/>
+      <c r="F18" s="34" t="n"/>
+      <c r="G18" s="34" t="n"/>
+      <c r="H18" s="34" t="n"/>
+      <c r="I18" s="34" t="n"/>
+      <c r="J18" s="34" t="n"/>
+      <c r="K18" s="34" t="n"/>
+      <c r="L18" s="34" t="n"/>
+      <c r="M18" s="34" t="n"/>
+      <c r="N18" s="34" t="n"/>
+    </row>
+    <row r="19" ht="15" customHeight="1" s="20">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>Revenue (€)</t>
+        </is>
+      </c>
+      <c r="B19" s="34" t="n"/>
+      <c r="C19" s="34" t="n"/>
+      <c r="D19" s="34" t="n"/>
+      <c r="E19" s="34" t="n"/>
+      <c r="F19" s="34" t="n"/>
+      <c r="G19" s="34" t="n"/>
+      <c r="H19" s="34" t="n"/>
+      <c r="I19" s="34" t="n"/>
+      <c r="J19" s="34" t="n"/>
+      <c r="K19" s="34" t="n"/>
+      <c r="L19" s="34" t="n"/>
+      <c r="M19" s="34" t="n"/>
+      <c r="N19" s="34" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>NPS (opinion)</t>
+        </is>
+      </c>
+      <c r="B20" s="34" t="n"/>
+      <c r="C20" s="34" t="n"/>
+      <c r="D20" s="34" t="n"/>
+      <c r="E20" s="34" t="n"/>
+      <c r="F20" s="34" t="n"/>
+      <c r="G20" s="34" t="n"/>
+      <c r="H20" s="34" t="n"/>
+      <c r="I20" s="34" t="n"/>
+      <c r="J20" s="34" t="n"/>
+      <c r="K20" s="34" t="n"/>
+      <c r="L20" s="34" t="n"/>
+      <c r="M20" s="34" t="n"/>
+      <c r="N20" s="34" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
+      <c r="I21" s="19" t="n"/>
+      <c r="J21" s="19" t="n"/>
+      <c r="K21" s="19" t="n"/>
+      <c r="L21" s="19" t="n"/>
+      <c r="M21" s="19" t="n"/>
+      <c r="N21" s="19" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>CUMULATIVE TOTALS</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
+      <c r="I22" s="19" t="n"/>
+      <c r="J22" s="19" t="n"/>
+      <c r="K22" s="19" t="n"/>
+      <c r="L22" s="19" t="n"/>
+      <c r="M22" s="19" t="n"/>
+      <c r="N22" s="19" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Total Interviews</t>
+        </is>
+      </c>
+      <c r="C23" s="35">
+        <f>SUM(B6:N6)</f>
+        <v/>
+      </c>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
+      <c r="I23" s="19" t="n"/>
+      <c r="J23" s="19" t="n"/>
+      <c r="K23" s="19" t="n"/>
+      <c r="L23" s="19" t="n"/>
+      <c r="M23" s="19" t="n"/>
+      <c r="N23" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Total Experiments</t>
+        </is>
+      </c>
+      <c r="C24" s="35">
+        <f>SUM(B7:N7)</f>
+        <v/>
+      </c>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
+      <c r="I24" s="19" t="n"/>
+      <c r="J24" s="19" t="n"/>
+      <c r="K24" s="19" t="n"/>
+      <c r="L24" s="19" t="n"/>
+      <c r="M24" s="19" t="n"/>
+      <c r="N24" s="19" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Total Revenue (€)</t>
+        </is>
+      </c>
+      <c r="C25" s="35">
+        <f>SUM(B19:N19)</f>
+        <v/>
+      </c>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
+      <c r="I25" s="19" t="n"/>
+      <c r="J25" s="19" t="n"/>
+      <c r="K25" s="19" t="n"/>
+      <c r="L25" s="19" t="n"/>
+      <c r="M25" s="19" t="n"/>
+      <c r="N25" s="19" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="C26" s="35">
+        <f>MAX(B15:N15)</f>
+        <v/>
+      </c>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
+      <c r="I26" s="19" t="n"/>
+      <c r="J26" s="19" t="n"/>
+      <c r="K26" s="19" t="n"/>
+      <c r="L26" s="19" t="n"/>
+      <c r="M26" s="19" t="n"/>
+      <c r="N26" s="19" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="19" t="n"/>
+      <c r="I27" s="19" t="n"/>
+      <c r="J27" s="19" t="n"/>
+      <c r="K27" s="19" t="n"/>
+      <c r="L27" s="19" t="n"/>
+      <c r="M27" s="19" t="n"/>
+      <c r="N27" s="19" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
+      <c r="I28" s="19" t="n"/>
+      <c r="J28" s="19" t="n"/>
+      <c r="K28" s="19" t="n"/>
+      <c r="L28" s="19" t="n"/>
+      <c r="M28" s="19" t="n"/>
+      <c r="N28" s="19" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="19" t="n"/>
+      <c r="I29" s="19" t="n"/>
+      <c r="J29" s="19" t="n"/>
+      <c r="K29" s="19" t="n"/>
+      <c r="L29" s="19" t="n"/>
+      <c r="M29" s="19" t="n"/>
+      <c r="N29" s="19" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
+      <c r="I30" s="19" t="n"/>
+      <c r="J30" s="19" t="n"/>
+      <c r="K30" s="19" t="n"/>
+      <c r="L30" s="19" t="n"/>
+      <c r="M30" s="19" t="n"/>
+      <c r="N30" s="19" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
+      <c r="I31" s="19" t="n"/>
+      <c r="J31" s="19" t="n"/>
+      <c r="K31" s="19" t="n"/>
+      <c r="L31" s="19" t="n"/>
+      <c r="M31" s="19" t="n"/>
+      <c r="N31" s="19" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="19" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="n"/>
+      <c r="H32" s="19" t="n"/>
+      <c r="I32" s="19" t="n"/>
+      <c r="J32" s="19" t="n"/>
+      <c r="K32" s="19" t="n"/>
+      <c r="L32" s="19" t="n"/>
+      <c r="M32" s="19" t="n"/>
+      <c r="N32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="19" t="n"/>
+      <c r="I33" s="19" t="n"/>
+      <c r="J33" s="19" t="n"/>
+      <c r="K33" s="19" t="n"/>
+      <c r="L33" s="19" t="n"/>
+      <c r="M33" s="19" t="n"/>
+      <c r="N33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="n"/>
+      <c r="H34" s="19" t="n"/>
+      <c r="I34" s="19" t="n"/>
+      <c r="J34" s="19" t="n"/>
+      <c r="K34" s="19" t="n"/>
+      <c r="L34" s="19" t="n"/>
+      <c r="M34" s="19" t="n"/>
+      <c r="N34" s="19" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="10" customWidth="1" style="19" min="1" max="1"/>
+    <col width="30.01" customWidth="1" style="19" min="2" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>WEEKLY REFLECTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="20">
+      <c r="A2" s="27" t="inlineStr">
+        <is>
+          <t>Complete each week before the next session</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="20">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>What were our 3 biggest learnings this week?</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>What assumptions did we validate or invalidate?</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>What surprised us most?</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>What's our riskiest assumption right now?</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>What's our #1 priority for next week?</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>What help do we need?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1" s="20">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>Module 00</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="n"/>
+      <c r="C5" s="36" t="n"/>
+      <c r="D5" s="36" t="n"/>
+      <c r="E5" s="36" t="n"/>
+      <c r="F5" s="36" t="n"/>
+      <c r="G5" s="36" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1" s="20">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>Module 01</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="n"/>
+      <c r="C6" s="36" t="n"/>
+      <c r="D6" s="36" t="n"/>
+      <c r="E6" s="36" t="n"/>
+      <c r="F6" s="36" t="n"/>
+      <c r="G6" s="36" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1" s="20">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>Module 02</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="n"/>
+      <c r="C7" s="36" t="n"/>
+      <c r="D7" s="36" t="n"/>
+      <c r="E7" s="36" t="n"/>
+      <c r="F7" s="36" t="n"/>
+      <c r="G7" s="36" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1" s="20">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>Module 03</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n"/>
+      <c r="C8" s="36" t="n"/>
+      <c r="D8" s="36" t="n"/>
+      <c r="E8" s="36" t="n"/>
+      <c r="F8" s="36" t="n"/>
+      <c r="G8" s="36" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1" s="20">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Module 04</t>
+        </is>
+      </c>
+      <c r="B9" s="36" t="n"/>
+      <c r="C9" s="36" t="n"/>
+      <c r="D9" s="36" t="n"/>
+      <c r="E9" s="36" t="n"/>
+      <c r="F9" s="36" t="n"/>
+      <c r="G9" s="36" t="n"/>
+    </row>
+    <row r="10" ht="60" customHeight="1" s="20">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>Module 05</t>
+        </is>
+      </c>
+      <c r="B10" s="36" t="n"/>
+      <c r="C10" s="36" t="n"/>
+      <c r="D10" s="36" t="n"/>
+      <c r="E10" s="36" t="n"/>
+      <c r="F10" s="36" t="n"/>
+      <c r="G10" s="36" t="n"/>
+    </row>
+    <row r="11" ht="60" customHeight="1" s="20">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>Module 06</t>
+        </is>
+      </c>
+      <c r="B11" s="36" t="n"/>
+      <c r="C11" s="36" t="n"/>
+      <c r="D11" s="36" t="n"/>
+      <c r="E11" s="36" t="n"/>
+      <c r="F11" s="36" t="n"/>
+      <c r="G11" s="36" t="n"/>
+    </row>
+    <row r="12" ht="60" customHeight="1" s="20">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>Module 07</t>
+        </is>
+      </c>
+      <c r="B12" s="36" t="n"/>
+      <c r="C12" s="36" t="n"/>
+      <c r="D12" s="36" t="n"/>
+      <c r="E12" s="36" t="n"/>
+      <c r="F12" s="36" t="n"/>
+      <c r="G12" s="36" t="n"/>
+    </row>
+    <row r="13" ht="60" customHeight="1" s="20">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>Module 08</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="36" t="n"/>
+      <c r="D13" s="36" t="n"/>
+      <c r="E13" s="36" t="n"/>
+      <c r="F13" s="36" t="n"/>
+      <c r="G13" s="36" t="n"/>
+    </row>
+    <row r="14" ht="60" customHeight="1" s="20">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>Module 09</t>
+        </is>
+      </c>
+      <c r="B14" s="36" t="n"/>
+      <c r="C14" s="36" t="n"/>
+      <c r="D14" s="36" t="n"/>
+      <c r="E14" s="36" t="n"/>
+      <c r="F14" s="36" t="n"/>
+      <c r="G14" s="36" t="n"/>
+    </row>
+    <row r="15" ht="60" customHeight="1" s="20">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>Module 10</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n"/>
+      <c r="C15" s="36" t="n"/>
+      <c r="D15" s="36" t="n"/>
+      <c r="E15" s="36" t="n"/>
+      <c r="F15" s="36" t="n"/>
+      <c r="G15" s="36" t="n"/>
+    </row>
+    <row r="16" ht="60" customHeight="1" s="20">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>Module 11</t>
+        </is>
+      </c>
+      <c r="B16" s="36" t="n"/>
+      <c r="C16" s="36" t="n"/>
+      <c r="D16" s="36" t="n"/>
+      <c r="E16" s="36" t="n"/>
+      <c r="F16" s="36" t="n"/>
+      <c r="G16" s="36" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>Module 12</t>
+        </is>
+      </c>
+      <c r="B17" s="36" t="n"/>
+      <c r="C17" s="36" t="n"/>
+      <c r="D17" s="36" t="n"/>
+      <c r="E17" s="36" t="n"/>
+      <c r="F17" s="36" t="n"/>
+      <c r="G17" s="36" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1372,7 +2493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1559,7 +2680,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1729,7 +2850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1785,6 +2906,107 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="20" min="1" max="1"/>
+    <col width="26" customWidth="1" style="20" min="2" max="2"/>
+    <col width="36" customWidth="1" style="20" min="3" max="3"/>
+    <col width="10" customWidth="1" style="20" min="4" max="4"/>
+    <col width="14" customWidth="1" style="20" min="5" max="5"/>
+    <col width="12" customWidth="1" style="20" min="6" max="6"/>
+    <col width="20" customWidth="1" style="20" min="7" max="7"/>
+    <col width="26" customWidth="1" style="20" min="8" max="8"/>
+    <col width="10" customWidth="1" style="20" min="9" max="9"/>
+    <col width="26" customWidth="1" style="20" min="10" max="10"/>
+    <col width="20" customWidth="1" style="20" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Module 07. One row per verdict. Crossed Kill Criteria Log lines decide first, then score framework 03's nine questions 0 to 2, each on an artifact. Provisional until the monkey test has run, confirmed at the Module 08 check-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1" s="20">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Crossed lines (Kill Criteria Log rows)</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Scores, questions 1 to 9 (0-2, with artifact)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Total (of 18)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Verdict (Go, Pivot, Kill)</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Pivot type (1, 2)</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Status (provisional, confirmed at Module 08)</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Named people (10)</t>
+        </is>
+      </c>
+      <c r="K4" s="28" t="inlineStr">
+        <is>
+          <t>Kill page (link)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3231,7 +4453,7 @@
     <row r="4" ht="15" customHeight="1" s="20">
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Methods: Interview, Survey, Landing Page, Click dummy, Prototype, Ad Test, Pricing Test</t>
+          <t>Methods: Interview, Survey, Landing Page, Click dummy, Prototype, Ad Test, Pricing Test (unit, price, structure, line in the Kill Criteria Log), Retention line (Kill Criteria Log row, read from the product's records)</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
@@ -4091,587 +5313,292 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" style="19" min="1" max="1"/>
-    <col width="8" customWidth="1" style="19" min="2" max="13"/>
-    <col width="13" customWidth="1" style="20" min="13" max="13"/>
-    <col width="13" customWidth="1" style="20" min="14" max="14"/>
+    <col width="12" customWidth="1" style="20" min="1" max="1"/>
+    <col width="10" customWidth="1" style="20" min="2" max="2"/>
+    <col width="18" customWidth="1" style="20" min="3" max="3"/>
+    <col width="22" customWidth="1" style="20" min="4" max="4"/>
+    <col width="14" customWidth="1" style="20" min="5" max="5"/>
+    <col width="16" customWidth="1" style="20" min="6" max="6"/>
+    <col width="26" customWidth="1" style="20" min="7" max="7"/>
+    <col width="14" customWidth="1" style="20" min="8" max="8"/>
+    <col width="14" customWidth="1" style="20" min="9" max="9"/>
+    <col width="18" customWidth="1" style="20" min="10" max="10"/>
+    <col width="30" customWidth="1" style="20" min="11" max="11"/>
+    <col width="20" customWidth="1" style="20" min="12" max="12"/>
+    <col width="20" customWidth="1" style="20" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
+    <row r="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>KPI TRACKER</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="20">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>WEEKLY METRICS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="20">
-      <c r="A4" s="32" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B4" s="32" t="inlineStr">
-        <is>
-          <t>M00</t>
-        </is>
-      </c>
-      <c r="C4" s="32" t="inlineStr">
-        <is>
-          <t>M01</t>
-        </is>
-      </c>
-      <c r="D4" s="32" t="inlineStr">
-        <is>
-          <t>M02</t>
-        </is>
-      </c>
-      <c r="E4" s="32" t="inlineStr">
-        <is>
-          <t>M03</t>
-        </is>
-      </c>
-      <c r="F4" s="32" t="inlineStr">
-        <is>
-          <t>M04</t>
-        </is>
-      </c>
-      <c r="G4" s="32" t="inlineStr">
-        <is>
-          <t>M05</t>
-        </is>
-      </c>
-      <c r="H4" s="32" t="inlineStr">
-        <is>
-          <t>M06</t>
-        </is>
-      </c>
-      <c r="I4" s="32" t="inlineStr">
-        <is>
-          <t>M07</t>
-        </is>
-      </c>
-      <c r="J4" s="32" t="inlineStr">
-        <is>
-          <t>M08</t>
-        </is>
-      </c>
-      <c r="K4" s="32" t="inlineStr">
-        <is>
-          <t>M09</t>
-        </is>
-      </c>
-      <c r="L4" s="32" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
-      </c>
-      <c r="M4" s="32" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
-      </c>
-      <c r="N4" s="32" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="20">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>Interviews Conducted</t>
-        </is>
-      </c>
-      <c r="B5" s="34" t="n"/>
-      <c r="C5" s="34" t="n"/>
-      <c r="D5" s="34" t="n"/>
-      <c r="E5" s="34" t="n"/>
-      <c r="F5" s="34" t="n"/>
-      <c r="G5" s="34" t="n"/>
-      <c r="H5" s="34" t="n"/>
-      <c r="I5" s="34" t="n"/>
-      <c r="J5" s="34" t="n"/>
-      <c r="K5" s="34" t="n"/>
-      <c r="L5" s="34" t="n"/>
-      <c r="M5" s="34" t="n"/>
-      <c r="N5" s="34" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="20">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>Experiments Run</t>
-        </is>
-      </c>
-      <c r="B6" s="34" t="n"/>
-      <c r="C6" s="34" t="n"/>
-      <c r="D6" s="34" t="n"/>
-      <c r="E6" s="34" t="n"/>
-      <c r="F6" s="34" t="n"/>
-      <c r="G6" s="34" t="n"/>
-      <c r="H6" s="34" t="n"/>
-      <c r="I6" s="34" t="n"/>
-      <c r="J6" s="34" t="n"/>
-      <c r="K6" s="34" t="n"/>
-      <c r="L6" s="34" t="n"/>
-      <c r="M6" s="34" t="n"/>
-      <c r="N6" s="34" t="n"/>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="20">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>Landing Page Visitors</t>
-        </is>
-      </c>
-      <c r="B7" s="34" t="n"/>
-      <c r="C7" s="34" t="n"/>
-      <c r="D7" s="34" t="n"/>
-      <c r="E7" s="34" t="n"/>
-      <c r="F7" s="34" t="n"/>
-      <c r="G7" s="34" t="n"/>
-      <c r="H7" s="34" t="n"/>
-      <c r="I7" s="34" t="n"/>
-      <c r="J7" s="34" t="n"/>
-      <c r="K7" s="34" t="n"/>
-      <c r="L7" s="34" t="n"/>
-      <c r="M7" s="34" t="n"/>
-      <c r="N7" s="34" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="20">
-      <c r="A8" s="33" t="inlineStr">
-        <is>
-          <t>Sign-ups / Leads</t>
-        </is>
-      </c>
-      <c r="B8" s="34" t="n"/>
-      <c r="C8" s="34" t="n"/>
-      <c r="D8" s="34" t="n"/>
-      <c r="E8" s="34" t="n"/>
-      <c r="F8" s="34" t="n"/>
-      <c r="G8" s="34" t="n"/>
-      <c r="H8" s="34" t="n"/>
-      <c r="I8" s="34" t="n"/>
-      <c r="J8" s="34" t="n"/>
-      <c r="K8" s="34" t="n"/>
-      <c r="L8" s="34" t="n"/>
-      <c r="M8" s="34" t="n"/>
-      <c r="N8" s="34" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="20">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>Prototype Users</t>
-        </is>
-      </c>
-      <c r="B9" s="34" t="n"/>
-      <c r="C9" s="34" t="n"/>
-      <c r="D9" s="34" t="n"/>
-      <c r="E9" s="34" t="n"/>
-      <c r="F9" s="34" t="n"/>
-      <c r="G9" s="34" t="n"/>
-      <c r="H9" s="34" t="n"/>
-      <c r="I9" s="34" t="n"/>
-      <c r="J9" s="34" t="n"/>
-      <c r="K9" s="34" t="n"/>
-      <c r="L9" s="34" t="n"/>
-      <c r="M9" s="34" t="n"/>
-      <c r="N9" s="34" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="20">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>Active Users (weekly)</t>
-        </is>
-      </c>
-      <c r="B10" s="34" t="n"/>
-      <c r="C10" s="34" t="n"/>
-      <c r="D10" s="34" t="n"/>
-      <c r="E10" s="34" t="n"/>
-      <c r="F10" s="34" t="n"/>
-      <c r="G10" s="34" t="n"/>
-      <c r="H10" s="34" t="n"/>
-      <c r="I10" s="34" t="n"/>
-      <c r="J10" s="34" t="n"/>
-      <c r="K10" s="34" t="n"/>
-      <c r="L10" s="34" t="n"/>
-      <c r="M10" s="34" t="n"/>
-      <c r="N10" s="34" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="20">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>Paying Customers</t>
-        </is>
-      </c>
-      <c r="B11" s="34" t="n"/>
-      <c r="C11" s="34" t="n"/>
-      <c r="D11" s="34" t="n"/>
-      <c r="E11" s="34" t="n"/>
-      <c r="F11" s="34" t="n"/>
-      <c r="G11" s="34" t="n"/>
-      <c r="H11" s="34" t="n"/>
-      <c r="I11" s="34" t="n"/>
-      <c r="J11" s="34" t="n"/>
-      <c r="K11" s="34" t="n"/>
-      <c r="L11" s="34" t="n"/>
-      <c r="M11" s="34" t="n"/>
-      <c r="N11" s="34" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="20">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>Revenue (€)</t>
-        </is>
-      </c>
-      <c r="B12" s="34" t="n"/>
-      <c r="C12" s="34" t="n"/>
-      <c r="D12" s="34" t="n"/>
-      <c r="E12" s="34" t="n"/>
-      <c r="F12" s="34" t="n"/>
-      <c r="G12" s="34" t="n"/>
-      <c r="H12" s="34" t="n"/>
-      <c r="I12" s="34" t="n"/>
-      <c r="J12" s="34" t="n"/>
-      <c r="K12" s="34" t="n"/>
-      <c r="L12" s="34" t="n"/>
-      <c r="M12" s="34" t="n"/>
-      <c r="N12" s="34" t="n"/>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="20">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>NPS Score</t>
-        </is>
-      </c>
-      <c r="B13" s="34" t="n"/>
-      <c r="C13" s="34" t="n"/>
-      <c r="D13" s="34" t="n"/>
-      <c r="E13" s="34" t="n"/>
-      <c r="F13" s="34" t="n"/>
-      <c r="G13" s="34" t="n"/>
-      <c r="H13" s="34" t="n"/>
-      <c r="I13" s="34" t="n"/>
-      <c r="J13" s="34" t="n"/>
-      <c r="K13" s="34" t="n"/>
-      <c r="L13" s="34" t="n"/>
-      <c r="M13" s="34" t="n"/>
-      <c r="N13" s="34" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="20">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t>CUMULATIVE TOTALS</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="20">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Total Interviews</t>
-        </is>
-      </c>
-      <c r="C16" s="35">
-        <f>SUM(B5:N5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="20">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>Total Experiments</t>
-        </is>
-      </c>
-      <c r="C17" s="35">
-        <f>SUM(B6:N6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="20">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>Total Revenue (€)</t>
-        </is>
-      </c>
-      <c r="C18" s="35">
-        <f>SUM(B12:N12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="20">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Total Customers</t>
-        </is>
-      </c>
-      <c r="C19" s="35">
-        <f>MAX(B11:N11)</f>
-        <v/>
+          <t>USE LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Module 06. One row per user of your live MVP. Watch them use it without your help. Only people from your segment count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1" s="20">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Date first used</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>User (name)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Role and segment</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Segment? (yes, mixed, no)</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>Brought by (student)</t>
+        </is>
+      </c>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Came from (first buyer, sign-up, interviewee, group, other)</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Used without help? (yes, no)</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Reached the outcome? (yes, no)</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Came back unprompted (date or no)</t>
+        </is>
+      </c>
+      <c r="K4" s="28" t="inlineStr">
+        <is>
+          <t>What stopped them</t>
+        </is>
+      </c>
+      <c r="L4" s="28" t="inlineStr">
+        <is>
+          <t>Fix shipped (version, date)</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="inlineStr">
+        <is>
+          <t>Asked to pay? (answer)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:X4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="19" min="1" max="1"/>
-    <col width="30.01" customWidth="1" style="19" min="2" max="7"/>
+    <col width="16" customWidth="1" style="20" min="1" max="1"/>
+    <col width="16" customWidth="1" style="20" min="2" max="2"/>
+    <col width="16" customWidth="1" style="20" min="3" max="3"/>
+    <col width="16" customWidth="1" style="20" min="4" max="4"/>
+    <col width="28" customWidth="1" style="20" min="5" max="5"/>
+    <col width="16" customWidth="1" style="20" min="6" max="6"/>
+    <col width="16" customWidth="1" style="20" min="7" max="7"/>
+    <col width="16" customWidth="1" style="20" min="8" max="8"/>
+    <col width="16" customWidth="1" style="20" min="9" max="9"/>
+    <col width="16" customWidth="1" style="20" min="10" max="10"/>
+    <col width="28" customWidth="1" style="20" min="11" max="11"/>
+    <col width="16" customWidth="1" style="20" min="12" max="12"/>
+    <col width="16" customWidth="1" style="20" min="13" max="13"/>
+    <col width="16" customWidth="1" style="20" min="14" max="14"/>
+    <col width="16" customWidth="1" style="20" min="15" max="15"/>
+    <col width="16" customWidth="1" style="20" min="16" max="16"/>
+    <col width="16" customWidth="1" style="20" min="17" max="17"/>
+    <col width="16" customWidth="1" style="20" min="18" max="18"/>
+    <col width="16" customWidth="1" style="20" min="19" max="19"/>
+    <col width="28" customWidth="1" style="20" min="20" max="20"/>
+    <col width="28" customWidth="1" style="20" min="21" max="21"/>
+    <col width="16" customWidth="1" style="20" min="22" max="22"/>
+    <col width="16" customWidth="1" style="20" min="23" max="23"/>
+    <col width="28" customWidth="1" style="20" min="24" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="20">
+    <row r="1">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>WEEKLY REFLECTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="20">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Complete each week before the next session</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="20">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>Module</t>
+          <t>PIPELINE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Module 08 and 09. One row per named person asked, then per payment. Only payments from outside your social graph count toward the bar. Proof is a dashboard screenshot or a paid numbered invoice, with names and bank details cropped before you show it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1" s="20">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Date</t>
         </is>
       </c>
       <c r="B4" s="28" t="inlineStr">
         <is>
-          <t>What were our 3 biggest learnings this week?</t>
+          <t>Person (name)</t>
         </is>
       </c>
       <c r="C4" s="28" t="inlineStr">
         <is>
-          <t>What assumptions did we validate or invalidate?</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="D4" s="28" t="inlineStr">
         <is>
-          <t>What surprised us most?</t>
+          <t>Segment</t>
         </is>
       </c>
       <c r="E4" s="28" t="inlineStr">
         <is>
-          <t>What's our riskiest assumption right now?</t>
+          <t>Source (Module 07 list, buyer, Use Log user, sign-up, interviewee, referral, new)</t>
         </is>
       </c>
       <c r="F4" s="28" t="inlineStr">
         <is>
-          <t>What's our #1 priority for next week?</t>
+          <t>Channel</t>
         </is>
       </c>
       <c r="G4" s="28" t="inlineStr">
         <is>
-          <t>What help do we need?</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1" s="20">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>Module 00</t>
-        </is>
-      </c>
-      <c r="B5" s="36" t="n"/>
-      <c r="C5" s="36" t="n"/>
-      <c r="D5" s="36" t="n"/>
-      <c r="E5" s="36" t="n"/>
-      <c r="F5" s="36" t="n"/>
-      <c r="G5" s="36" t="n"/>
-    </row>
-    <row r="6" ht="60" customHeight="1" s="20">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="B6" s="36" t="n"/>
-      <c r="C6" s="36" t="n"/>
-      <c r="D6" s="36" t="n"/>
-      <c r="E6" s="36" t="n"/>
-      <c r="F6" s="36" t="n"/>
-      <c r="G6" s="36" t="n"/>
-    </row>
-    <row r="7" ht="60" customHeight="1" s="20">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>Module 02</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="n"/>
-      <c r="C7" s="36" t="n"/>
-      <c r="D7" s="36" t="n"/>
-      <c r="E7" s="36" t="n"/>
-      <c r="F7" s="36" t="n"/>
-      <c r="G7" s="36" t="n"/>
-    </row>
-    <row r="8" ht="60" customHeight="1" s="20">
-      <c r="A8" s="33" t="inlineStr">
-        <is>
-          <t>Module 03</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="n"/>
-      <c r="C8" s="36" t="n"/>
-      <c r="D8" s="36" t="n"/>
-      <c r="E8" s="36" t="n"/>
-      <c r="F8" s="36" t="n"/>
-      <c r="G8" s="36" t="n"/>
-    </row>
-    <row r="9" ht="60" customHeight="1" s="20">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>Module 04</t>
-        </is>
-      </c>
-      <c r="B9" s="36" t="n"/>
-      <c r="C9" s="36" t="n"/>
-      <c r="D9" s="36" t="n"/>
-      <c r="E9" s="36" t="n"/>
-      <c r="F9" s="36" t="n"/>
-      <c r="G9" s="36" t="n"/>
-    </row>
-    <row r="10" ht="60" customHeight="1" s="20">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>Module 05</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n"/>
-      <c r="C10" s="36" t="n"/>
-      <c r="D10" s="36" t="n"/>
-      <c r="E10" s="36" t="n"/>
-      <c r="F10" s="36" t="n"/>
-      <c r="G10" s="36" t="n"/>
-    </row>
-    <row r="11" ht="60" customHeight="1" s="20">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>Module 06</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n"/>
-      <c r="C11" s="36" t="n"/>
-      <c r="D11" s="36" t="n"/>
-      <c r="E11" s="36" t="n"/>
-      <c r="F11" s="36" t="n"/>
-      <c r="G11" s="36" t="n"/>
-    </row>
-    <row r="12" ht="60" customHeight="1" s="20">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>Module 07</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n"/>
-      <c r="C12" s="36" t="n"/>
-      <c r="D12" s="36" t="n"/>
-      <c r="E12" s="36" t="n"/>
-      <c r="F12" s="36" t="n"/>
-      <c r="G12" s="36" t="n"/>
-    </row>
-    <row r="13" ht="60" customHeight="1" s="20">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>Module 08</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="n"/>
-      <c r="C13" s="36" t="n"/>
-      <c r="D13" s="36" t="n"/>
-      <c r="E13" s="36" t="n"/>
-      <c r="F13" s="36" t="n"/>
-      <c r="G13" s="36" t="n"/>
-    </row>
-    <row r="14" ht="60" customHeight="1" s="20">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>Module 09</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="n"/>
-      <c r="C14" s="36" t="n"/>
-      <c r="D14" s="36" t="n"/>
-      <c r="E14" s="36" t="n"/>
-      <c r="F14" s="36" t="n"/>
-      <c r="G14" s="36" t="n"/>
-    </row>
-    <row r="15" ht="60" customHeight="1" s="20">
-      <c r="A15" s="33" t="inlineStr">
-        <is>
-          <t>Module 10</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="n"/>
-      <c r="C15" s="36" t="n"/>
-      <c r="D15" s="36" t="n"/>
-      <c r="E15" s="36" t="n"/>
-      <c r="F15" s="36" t="n"/>
-      <c r="G15" s="36" t="n"/>
-    </row>
-    <row r="16" ht="60" customHeight="1" s="20">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>Module 11</t>
-        </is>
-      </c>
-      <c r="B16" s="36" t="n"/>
-      <c r="C16" s="36" t="n"/>
-      <c r="D16" s="36" t="n"/>
-      <c r="E16" s="36" t="n"/>
-      <c r="F16" s="36" t="n"/>
-      <c r="G16" s="36" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>Module 12</t>
-        </is>
-      </c>
-      <c r="B17" s="36" t="n"/>
-      <c r="C17" s="36" t="n"/>
-      <c r="D17" s="36" t="n"/>
-      <c r="E17" s="36" t="n"/>
-      <c r="F17" s="36" t="n"/>
-      <c r="G17" s="36" t="n"/>
+          <t>Brought by (founder)</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Touches (dates)</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Reply (yes, no, none)</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Call held (date)</t>
+        </is>
+      </c>
+      <c r="K4" s="28" t="inlineStr">
+        <is>
+          <t>Activated (yes, no, from the Use Log)</t>
+        </is>
+      </c>
+      <c r="L4" s="28" t="inlineStr">
+        <is>
+          <t>Offer and price asked</t>
+        </is>
+      </c>
+      <c r="M4" s="28" t="inlineStr">
+        <is>
+          <t>Sent to the price (date)</t>
+        </is>
+      </c>
+      <c r="N4" s="28" t="inlineStr">
+        <is>
+          <t>Answer (paid, yes, no, later)</t>
+        </is>
+      </c>
+      <c r="O4" s="28" t="inlineStr">
+        <is>
+          <t>Objection, word for word</t>
+        </is>
+      </c>
+      <c r="P4" s="28" t="inlineStr">
+        <is>
+          <t>Objection category</t>
+        </is>
+      </c>
+      <c r="Q4" s="28" t="inlineStr">
+        <is>
+          <t>Paid on</t>
+        </is>
+      </c>
+      <c r="R4" s="28" t="inlineStr">
+        <is>
+          <t>Amount (€)</t>
+        </is>
+      </c>
+      <c r="S4" s="28" t="inlineStr">
+        <is>
+          <t>Through the product or by hand</t>
+        </is>
+      </c>
+      <c r="T4" s="28" t="inlineStr">
+        <is>
+          <t>Proof (screenshot link or invoice number)</t>
+        </is>
+      </c>
+      <c r="U4" s="28" t="inlineStr">
+        <is>
+          <t>Same offer bought again by another customer (yes, no)</t>
+        </is>
+      </c>
+      <c r="V4" s="28" t="inlineStr">
+        <is>
+          <t>Back on (used or paid, date)</t>
+        </is>
+      </c>
+      <c r="W4" s="28" t="inlineStr">
+        <is>
+          <t>Lost, reason in their words</t>
+        </is>
+      </c>
+      <c r="X4" s="28" t="inlineStr">
+        <is>
+          <t>Outside your social graph (yes, no)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:X1"/>
   </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Module 00 gets an evidence check: backup slides at the end of the lecture back its claims with research and data (an AI bubble test on the Nasdaq-100, how often big bets fail and how far they grow, and the mathematics of startup against small business), and several claims are corrected. The lecture decks of Modules 00, 02 to 05 and 10 open with the course path and a pivot-or-persevere checkpoint, with new step-by-step screenshots in Modules 04 and 10. Module 10 gets the new Tally case, which replaces Linear, and its separate slide decks leave. Updated glossary, grading rubric, reading list, team stack, Student Toolkit, default-alive calculator and deck design. New: Getting Help.
</commit_message>
<xml_diff>
--- a/resources/Student_Toolkit.xlsx
+++ b/resources/Student_Toolkit.xlsx
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B10" s="19">
-        <f>'KPI Tracker'!C25</f>
+        <f>'KPI Tracker'!C28</f>
         <v/>
       </c>
       <c r="C10" s="19" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B11" s="19">
-        <f>'KPI Tracker'!C26</f>
+        <f>'KPI Tracker'!C29</f>
         <v/>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1213,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="25" customWidth="1" style="19" min="1" max="1"/>
@@ -1611,7 +1611,7 @@
     <row r="20">
       <c r="A20" s="33" t="inlineStr">
         <is>
-          <t>NPS (opinion)</t>
+          <t>Burn (€ a month)</t>
         </is>
       </c>
       <c r="B20" s="34" t="n"/>
@@ -1629,71 +1629,69 @@
       <c r="N20" s="34" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-      <c r="E21" s="19" t="n"/>
-      <c r="F21" s="19" t="n"/>
-      <c r="G21" s="19" t="n"/>
-      <c r="H21" s="19" t="n"/>
-      <c r="I21" s="19" t="n"/>
-      <c r="J21" s="19" t="n"/>
-      <c r="K21" s="19" t="n"/>
-      <c r="L21" s="19" t="n"/>
-      <c r="M21" s="19" t="n"/>
-      <c r="N21" s="19" t="n"/>
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Cash (€)</t>
+        </is>
+      </c>
+      <c r="B21" s="34" t="n"/>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="34" t="n"/>
+      <c r="E21" s="34" t="n"/>
+      <c r="F21" s="34" t="n"/>
+      <c r="G21" s="34" t="n"/>
+      <c r="H21" s="34" t="n"/>
+      <c r="I21" s="34" t="n"/>
+      <c r="J21" s="34" t="n"/>
+      <c r="K21" s="34" t="n"/>
+      <c r="L21" s="34" t="n"/>
+      <c r="M21" s="34" t="n"/>
+      <c r="N21" s="34" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
-        <is>
-          <t>CUMULATIVE TOTALS</t>
-        </is>
-      </c>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="19" t="n"/>
-      <c r="F22" s="19" t="n"/>
-      <c r="G22" s="19" t="n"/>
-      <c r="H22" s="19" t="n"/>
-      <c r="I22" s="19" t="n"/>
-      <c r="J22" s="19" t="n"/>
-      <c r="K22" s="19" t="n"/>
-      <c r="L22" s="19" t="n"/>
-      <c r="M22" s="19" t="n"/>
-      <c r="N22" s="19" t="n"/>
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>Runway (months)</t>
+        </is>
+      </c>
+      <c r="B22" s="34" t="n"/>
+      <c r="C22" s="34" t="n"/>
+      <c r="D22" s="34" t="n"/>
+      <c r="E22" s="34" t="n"/>
+      <c r="F22" s="34" t="n"/>
+      <c r="G22" s="34" t="n"/>
+      <c r="H22" s="34" t="n"/>
+      <c r="I22" s="34" t="n"/>
+      <c r="J22" s="34" t="n"/>
+      <c r="K22" s="34" t="n"/>
+      <c r="L22" s="34" t="n"/>
+      <c r="M22" s="34" t="n"/>
+      <c r="N22" s="34" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>Total Interviews</t>
-        </is>
-      </c>
-      <c r="C23" s="35">
-        <f>SUM(B6:N6)</f>
-        <v/>
-      </c>
-      <c r="D23" s="19" t="n"/>
-      <c r="E23" s="19" t="n"/>
-      <c r="F23" s="19" t="n"/>
-      <c r="G23" s="19" t="n"/>
-      <c r="H23" s="19" t="n"/>
-      <c r="I23" s="19" t="n"/>
-      <c r="J23" s="19" t="n"/>
-      <c r="K23" s="19" t="n"/>
-      <c r="L23" s="19" t="n"/>
-      <c r="M23" s="19" t="n"/>
-      <c r="N23" s="19" t="n"/>
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>NPS (opinion)</t>
+        </is>
+      </c>
+      <c r="B23" s="34" t="n"/>
+      <c r="C23" s="34" t="n"/>
+      <c r="D23" s="34" t="n"/>
+      <c r="E23" s="34" t="n"/>
+      <c r="F23" s="34" t="n"/>
+      <c r="G23" s="34" t="n"/>
+      <c r="H23" s="34" t="n"/>
+      <c r="I23" s="34" t="n"/>
+      <c r="J23" s="34" t="n"/>
+      <c r="K23" s="34" t="n"/>
+      <c r="L23" s="34" t="n"/>
+      <c r="M23" s="34" t="n"/>
+      <c r="N23" s="34" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
-        <is>
-          <t>Total Experiments</t>
-        </is>
-      </c>
-      <c r="C24" s="35">
-        <f>SUM(B7:N7)</f>
-        <v/>
-      </c>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
       <c r="D24" s="19" t="n"/>
       <c r="E24" s="19" t="n"/>
       <c r="F24" s="19" t="n"/>
@@ -1707,14 +1705,10 @@
       <c r="N24" s="19" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>Total Revenue (€)</t>
-        </is>
-      </c>
-      <c r="C25" s="35">
-        <f>SUM(B19:N19)</f>
-        <v/>
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>CUMULATIVE TOTALS</t>
+        </is>
       </c>
       <c r="D25" s="19" t="n"/>
       <c r="E25" s="19" t="n"/>
@@ -1731,11 +1725,11 @@
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Total Customers</t>
+          <t>Total Interviews</t>
         </is>
       </c>
       <c r="C26" s="35">
-        <f>MAX(B15:N15)</f>
+        <f>SUM(B6:N6)</f>
         <v/>
       </c>
       <c r="D26" s="19" t="n"/>
@@ -1751,9 +1745,15 @@
       <c r="N26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="19" t="n"/>
-      <c r="C27" s="19" t="n"/>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Total Experiments</t>
+        </is>
+      </c>
+      <c r="C27" s="35">
+        <f>SUM(B7:N7)</f>
+        <v/>
+      </c>
       <c r="D27" s="19" t="n"/>
       <c r="E27" s="19" t="n"/>
       <c r="F27" s="19" t="n"/>
@@ -1767,9 +1767,15 @@
       <c r="N27" s="19" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="19" t="n"/>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Total Revenue (€)</t>
+        </is>
+      </c>
+      <c r="C28" s="35">
+        <f>SUM(B19:N19)</f>
+        <v/>
+      </c>
       <c r="D28" s="19" t="n"/>
       <c r="E28" s="19" t="n"/>
       <c r="F28" s="19" t="n"/>
@@ -1783,9 +1789,15 @@
       <c r="N28" s="19" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="19" t="n"/>
-      <c r="C29" s="19" t="n"/>
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Total Customers</t>
+        </is>
+      </c>
+      <c r="C29" s="35">
+        <f>MAX(B15:N15)</f>
+        <v/>
+      </c>
       <c r="D29" s="19" t="n"/>
       <c r="E29" s="19" t="n"/>
       <c r="F29" s="19" t="n"/>
@@ -1878,10 +1890,90 @@
       <c r="M34" s="19" t="n"/>
       <c r="N34" s="19" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="19" t="n"/>
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="19" t="n"/>
+      <c r="I35" s="19" t="n"/>
+      <c r="J35" s="19" t="n"/>
+      <c r="K35" s="19" t="n"/>
+      <c r="L35" s="19" t="n"/>
+      <c r="M35" s="19" t="n"/>
+      <c r="N35" s="19" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="19" t="n"/>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
+      <c r="I36" s="19" t="n"/>
+      <c r="J36" s="19" t="n"/>
+      <c r="K36" s="19" t="n"/>
+      <c r="L36" s="19" t="n"/>
+      <c r="M36" s="19" t="n"/>
+      <c r="N36" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="n"/>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
+      <c r="I37" s="19" t="n"/>
+      <c r="J37" s="19" t="n"/>
+      <c r="K37" s="19" t="n"/>
+      <c r="L37" s="19" t="n"/>
+      <c r="M37" s="19" t="n"/>
+      <c r="N37" s="19" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="19" t="n"/>
+      <c r="H38" s="19" t="n"/>
+      <c r="I38" s="19" t="n"/>
+      <c r="J38" s="19" t="n"/>
+      <c r="K38" s="19" t="n"/>
+      <c r="L38" s="19" t="n"/>
+      <c r="M38" s="19" t="n"/>
+      <c r="N38" s="19" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="19" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
+      <c r="I39" s="19" t="n"/>
+      <c r="J39" s="19" t="n"/>
+      <c r="K39" s="19" t="n"/>
+      <c r="L39" s="19" t="n"/>
+      <c r="M39" s="19" t="n"/>
+      <c r="N39" s="19" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A22:C22"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2499,46 +2591,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="44.99" customWidth="1" style="19" min="1" max="1"/>
-    <col width="8" customWidth="1" style="19" min="2" max="2"/>
+    <col width="70" customWidth="1" style="19" min="1" max="1"/>
+    <col width="22" customWidth="1" style="19" min="2" max="2"/>
     <col width="35" customWidth="1" style="19" min="3" max="3"/>
     <col width="30.01" customWidth="1" style="19" min="4" max="4"/>
+    <col width="30" customWidth="1" style="20" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="20">
       <c r="A1" s="25" t="inlineStr">
         <is>
-          <t>FINAL SUBMISSION CHECKLIST</t>
+          <t>EVIDENCE PACK</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="20">
       <c r="A2" s="27" t="inlineStr">
         <is>
-          <t>Check off items as you complete them</t>
-        </is>
-      </c>
-    </row>
+          <t>Your Toolkit as it stands is your evidence pack. Before Demo Day, check that each record exists and is current. Nothing here is handed in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="20">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>Required Deliverable</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B4" s="23" t="inlineStr">
         <is>
+          <t>Rubric dimension</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="inlineStr">
+        <is>
           <t>Done?</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
-        <is>
-          <t>Link/Location</t>
-        </is>
-      </c>
       <c r="D4" s="23" t="inlineStr">
+        <is>
+          <t>Link or sheet</t>
+        </is>
+      </c>
+      <c r="E4" s="23" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2547,132 +2646,164 @@
     <row r="5" ht="15" customHeight="1" s="20">
       <c r="A5" s="19" t="inlineStr">
         <is>
-          <t>Final pitch deck (updated with feedback)</t>
+          <t>Pipeline, each payment with its proof (dashboard screenshot or numbered invoice), outside your social graph</t>
         </is>
       </c>
       <c r="B5" s="37" t="inlineStr">
         <is>
+          <t>Verified traction</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n"/>
       <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="20">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Live demo recording link</t>
+          <t>Revenue Ladder, cumulative revenue by module</t>
         </is>
       </c>
       <c r="B6" s="37" t="inlineStr">
         <is>
+          <t>Verified traction</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n"/>
       <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="20">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>Prototype access (repo or share link)</t>
+          <t>Interview Log, a named contact and one verbatim quote per conversation</t>
         </is>
       </c>
       <c r="B7" s="37" t="inlineStr">
         <is>
+          <t>Evidence quality</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n"/>
       <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="20">
       <c r="A8" s="19" t="inlineStr">
         <is>
-          <t>Interview log (10-15/week documented)</t>
+          <t>Experiment Tracker and Traffic Sources, each test with its result</t>
         </is>
       </c>
       <c r="B8" s="37" t="inlineStr">
         <is>
+          <t>Evidence quality</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n"/>
       <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="20">
       <c r="A9" s="19" t="inlineStr">
         <is>
-          <t>Experiment tracker (all experiments)</t>
+          <t>Kill Criteria Log, every line dated before its test, with the result</t>
         </is>
       </c>
       <c r="B9" s="37" t="inlineStr">
         <is>
+          <t>Decision discipline</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n"/>
       <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="20">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>Analytics snapshot</t>
+          <t>Verdict, the Module 07 verdict and the verdict on the company after Demo Day</t>
         </is>
       </c>
       <c r="B10" s="37" t="inlineStr">
         <is>
+          <t>Decision discipline</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n"/>
       <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="20">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>KPI sheet with weekly data</t>
+          <t>KPI Tracker, weekly numbers including burn, cash and runway</t>
         </is>
       </c>
       <c r="B11" s="37" t="inlineStr">
         <is>
+          <t>Verified traction</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C11" s="22" t="n"/>
       <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="20">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>Individual reflection essay</t>
+          <t>Your pitch, ten slides in Sequoia's order or fewer</t>
         </is>
       </c>
       <c r="B12" s="37" t="inlineStr">
         <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
           <t>☐</t>
         </is>
       </c>
-      <c r="C12" s="22" t="n"/>
       <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="20">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>Team photo</t>
-        </is>
-      </c>
-      <c r="B13" s="37" t="inlineStr">
-        <is>
-          <t>☐</t>
-        </is>
-      </c>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="37" t="n"/>
       <c r="C13" s="22" t="n"/>
       <c r="D13" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2794,7 +2925,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>€1,000 verified minimum + evidence pack</t>
+          <t>€2,000 verified minimum + evidence pack</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
@@ -2979,7 +3110,7 @@
       </c>
       <c r="G4" s="28" t="inlineStr">
         <is>
-          <t>Status (provisional, confirmed at Module 08)</t>
+          <t>Status (provisional or confirmed, with date)</t>
         </is>
       </c>
       <c r="H4" s="28" t="inlineStr">
@@ -4011,7 +4142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="20" min="1" max="1"/>
@@ -4036,7 +4167,7 @@
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Module 01. Every founder confirms the agreement after the end-of-week feedback round. Revisit it on the review date.</t>
+          <t>Module 01. Every founder confirms the agreement after the end-of-week feedback round. Revisit it on the review date. Module 11 adds how you look after each other.</t>
         </is>
       </c>
     </row>
@@ -4177,24 +4308,73 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" s="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Feedback routine</t>
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" s="20">
       <c r="A21" s="19" t="inlineStr">
         <is>
-          <t>Review date</t>
+          <t>How we look after each other (Module 11): our check-in rhythm, time off, our team stop line, what we do when one of us struggles</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="19" t="inlineStr">
         <is>
+          <t>Review date</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
           <t>Changes after the end-of-week feedback round</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>After Demo Day: who does what, with how much time</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Next revenue target and its date</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Next kill line</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Who owns the code, the brand and the money</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Next outside meeting (who, date)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>Accountability group, next date</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="20" min="1" max="1"/>
@@ -5443,8 +5623,8 @@
     <col width="16" customWidth="1" style="20" min="8" max="8"/>
     <col width="16" customWidth="1" style="20" min="9" max="9"/>
     <col width="16" customWidth="1" style="20" min="10" max="10"/>
-    <col width="28" customWidth="1" style="20" min="11" max="11"/>
-    <col width="16" customWidth="1" style="20" min="12" max="12"/>
+    <col width="16" customWidth="1" style="20" min="11" max="11"/>
+    <col width="28" customWidth="1" style="20" min="12" max="12"/>
     <col width="16" customWidth="1" style="20" min="13" max="13"/>
     <col width="16" customWidth="1" style="20" min="14" max="14"/>
     <col width="16" customWidth="1" style="20" min="15" max="15"/>
@@ -5452,11 +5632,12 @@
     <col width="16" customWidth="1" style="20" min="17" max="17"/>
     <col width="16" customWidth="1" style="20" min="18" max="18"/>
     <col width="16" customWidth="1" style="20" min="19" max="19"/>
-    <col width="28" customWidth="1" style="20" min="20" max="20"/>
+    <col width="16" customWidth="1" style="20" min="20" max="20"/>
     <col width="28" customWidth="1" style="20" min="21" max="21"/>
-    <col width="16" customWidth="1" style="20" min="22" max="22"/>
+    <col width="28" customWidth="1" style="20" min="22" max="22"/>
     <col width="16" customWidth="1" style="20" min="23" max="23"/>
-    <col width="28" customWidth="1" style="20" min="24" max="24"/>
+    <col width="16" customWidth="1" style="20" min="24" max="24"/>
+    <col width="28" customWidth="1" style="20" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5516,80 +5697,85 @@
       </c>
       <c r="I4" s="28" t="inlineStr">
         <is>
+          <t>Next follow-up (date)</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
           <t>Reply (yes, no, none)</t>
         </is>
       </c>
-      <c r="J4" s="28" t="inlineStr">
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>Call held (date)</t>
         </is>
       </c>
-      <c r="K4" s="28" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr">
         <is>
           <t>Activated (yes, no, from the Use Log)</t>
         </is>
       </c>
-      <c r="L4" s="28" t="inlineStr">
+      <c r="M4" s="28" t="inlineStr">
         <is>
           <t>Offer and price asked</t>
         </is>
       </c>
-      <c r="M4" s="28" t="inlineStr">
+      <c r="N4" s="28" t="inlineStr">
         <is>
           <t>Sent to the price (date)</t>
         </is>
       </c>
-      <c r="N4" s="28" t="inlineStr">
+      <c r="O4" s="28" t="inlineStr">
         <is>
           <t>Answer (paid, yes, no, later)</t>
         </is>
       </c>
-      <c r="O4" s="28" t="inlineStr">
+      <c r="P4" s="28" t="inlineStr">
         <is>
           <t>Objection, word for word</t>
         </is>
       </c>
-      <c r="P4" s="28" t="inlineStr">
+      <c r="Q4" s="28" t="inlineStr">
         <is>
           <t>Objection category</t>
         </is>
       </c>
-      <c r="Q4" s="28" t="inlineStr">
+      <c r="R4" s="28" t="inlineStr">
         <is>
           <t>Paid on</t>
         </is>
       </c>
-      <c r="R4" s="28" t="inlineStr">
+      <c r="S4" s="28" t="inlineStr">
         <is>
           <t>Amount (€)</t>
         </is>
       </c>
-      <c r="S4" s="28" t="inlineStr">
+      <c r="T4" s="28" t="inlineStr">
         <is>
           <t>Through the product or by hand</t>
         </is>
       </c>
-      <c r="T4" s="28" t="inlineStr">
+      <c r="U4" s="28" t="inlineStr">
         <is>
           <t>Proof (screenshot link or invoice number)</t>
         </is>
       </c>
-      <c r="U4" s="28" t="inlineStr">
+      <c r="V4" s="28" t="inlineStr">
         <is>
           <t>Same offer bought again by another customer (yes, no)</t>
         </is>
       </c>
-      <c r="V4" s="28" t="inlineStr">
+      <c r="W4" s="28" t="inlineStr">
         <is>
           <t>Back on (used or paid, date)</t>
         </is>
       </c>
-      <c r="W4" s="28" t="inlineStr">
+      <c r="X4" s="28" t="inlineStr">
         <is>
           <t>Lost, reason in their words</t>
         </is>
       </c>
-      <c r="X4" s="28" t="inlineStr">
+      <c r="Y4" s="28" t="inlineStr">
         <is>
           <t>Outside your social graph (yes, no)</t>
         </is>
@@ -5597,7 +5783,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:X1"/>
+    <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>